<commit_message>
changes in laptop (ignore)
</commit_message>
<xml_diff>
--- a/data/Coupling Config.xlsx
+++ b/data/Coupling Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\toolbox-amiris-emlab\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E072CA81-68EA-48A0-B202-BC1E5BEDA740}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38A03C84-272F-4942-A814-2F1FAC51E40E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="1" xr2:uid="{0615D95F-70E0-4B73-ABCC-D3A4B52943C0}"/>
   </bookViews>
@@ -1100,7 +1100,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="10">
-        <v>2050</v>
+        <v>2029</v>
       </c>
       <c r="E3" s="4">
         <f>2050+6</f>
@@ -1112,7 +1112,7 @@
         <v>80</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>96</v>

</xml_diff>